<commit_message>
updates and add one site_specific
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2074" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57EBF10D-1A7B-4961-BD3D-623461D58D43}"/>
+  <xr:revisionPtr revIDLastSave="2091" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1436FE9-8ACE-4EC7-AEBE-5D7830C85E4F}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="-26820" yWindow="1695" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2193" uniqueCount="801">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2207" uniqueCount="805">
   <si>
     <t>Durham</t>
   </si>
@@ -2413,9 +2413,6 @@
     <t>Gray</t>
   </si>
   <si>
-    <t xml:space="preserve">no reporting </t>
-  </si>
-  <si>
     <t xml:space="preserve">Souther Portland </t>
   </si>
   <si>
@@ -2441,6 +2438,21 @@
   </si>
   <si>
     <t>H:\BRWM\PFAS - LD 1600\Sites\New Gloucester\H Johnston S-021541 New Gloucester</t>
+  </si>
+  <si>
+    <t xml:space="preserve">South Portland </t>
+  </si>
+  <si>
+    <t>H:\BRWM\Remediation Division\Sites\Portland\Portland Harbor Dredge Project</t>
+  </si>
+  <si>
+    <t>SP Harbor Dredge</t>
+  </si>
+  <si>
+    <t>L2656748-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not reporting </t>
   </si>
 </sst>
 </file>
@@ -6961,7 +6973,9 @@
       <c r="A121" s="3" t="s">
         <v>588</v>
       </c>
-      <c r="B121" s="30"/>
+      <c r="B121" s="30" t="s">
+        <v>803</v>
+      </c>
       <c r="C121" s="3" t="s">
         <v>388</v>
       </c>
@@ -6971,18 +6985,28 @@
       <c r="E121" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
-      <c r="H121" s="4"/>
-      <c r="I121" s="4"/>
-      <c r="J121" s="4"/>
+      <c r="F121" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G121" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H121" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I121" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="J121" s="4" t="s">
+        <v>783</v>
+      </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
         <v>588</v>
       </c>
       <c r="B122" s="30" t="s">
-        <v>797</v>
+        <v>796</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>788</v>
@@ -7009,7 +7033,7 @@
         <v>783</v>
       </c>
       <c r="K122" s="23" t="s">
-        <v>791</v>
+        <v>804</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
@@ -7017,10 +7041,10 @@
         <v>22</v>
       </c>
       <c r="B123" s="30" t="s">
+        <v>794</v>
+      </c>
+      <c r="C123" s="3" t="s">
         <v>795</v>
-      </c>
-      <c r="C123" s="3" t="s">
-        <v>796</v>
       </c>
       <c r="D123" s="34">
         <v>46247</v>
@@ -7330,7 +7354,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -8892,6 +8916,9 @@
       <c r="H48" s="9" t="s">
         <v>498</v>
       </c>
+      <c r="J48" t="s">
+        <v>529</v>
+      </c>
       <c r="K48">
         <v>373157</v>
       </c>
@@ -10611,10 +10638,10 @@
         <v>88</v>
       </c>
       <c r="B103" s="17" t="s">
+        <v>791</v>
+      </c>
+      <c r="C103" s="13" t="s">
         <v>792</v>
-      </c>
-      <c r="C103" s="13" t="s">
-        <v>793</v>
       </c>
       <c r="D103" t="s">
         <v>88</v>
@@ -10623,7 +10650,7 @@
         <v>726</v>
       </c>
       <c r="F103" t="s">
-        <v>794</v>
+        <v>793</v>
       </c>
       <c r="K103">
         <v>395950</v>
@@ -10637,10 +10664,10 @@
         <v>29148</v>
       </c>
       <c r="B104" s="17" t="s">
+        <v>797</v>
+      </c>
+      <c r="C104" s="13" t="s">
         <v>798</v>
-      </c>
-      <c r="C104" s="13" t="s">
-        <v>799</v>
       </c>
       <c r="D104" t="s">
         <v>88</v>
@@ -10652,13 +10679,36 @@
         <v>755</v>
       </c>
       <c r="I104" s="9" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="K104">
         <v>399074</v>
       </c>
       <c r="L104">
         <v>4870081</v>
+      </c>
+    </row>
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>88</v>
+      </c>
+      <c r="B105" s="17" t="s">
+        <v>800</v>
+      </c>
+      <c r="C105" s="13" t="s">
+        <v>802</v>
+      </c>
+      <c r="D105" t="s">
+        <v>88</v>
+      </c>
+      <c r="E105" t="s">
+        <v>225</v>
+      </c>
+      <c r="F105" t="s">
+        <v>456</v>
+      </c>
+      <c r="I105" s="9" t="s">
+        <v>801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates and add common geology file parsing to pfas_table_edd
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2091" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1436FE9-8ACE-4EC7-AEBE-5D7830C85E4F}"/>
+  <xr:revisionPtr revIDLastSave="2101" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7FB35F1-1DC2-428C-B386-991C590E2971}"/>
   <bookViews>
-    <workbookView xWindow="-26820" yWindow="1695" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="3345" yWindow="4395" windowWidth="21600" windowHeight="11295" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2207" uniqueCount="805">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2217" uniqueCount="808">
   <si>
     <t>Durham</t>
   </si>
@@ -2453,6 +2453,15 @@
   </si>
   <si>
     <t xml:space="preserve">not reporting </t>
+  </si>
+  <si>
+    <t>FieldT1</t>
+  </si>
+  <si>
+    <t>DACF soil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L2636014-01 </t>
   </si>
 </sst>
 </file>
@@ -7069,15 +7078,37 @@
       </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A124" s="3"/>
-      <c r="B124" s="30"/>
+      <c r="A124" s="3" t="s">
+        <v>584</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>807</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>805</v>
+      </c>
       <c r="D124" s="34"/>
-      <c r="E124" s="4"/>
-      <c r="F124" s="4"/>
-      <c r="G124" s="4"/>
-      <c r="H124" s="4"/>
-      <c r="I124" s="4"/>
-      <c r="J124" s="4"/>
+      <c r="E124" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="F124" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="G124" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="H124" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="I124" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="J124" s="4" t="s">
+        <v>783</v>
+      </c>
+      <c r="K124" s="23" t="s">
+        <v>806</v>
+      </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125" s="3"/>
@@ -11777,6 +11808,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100125872C61801B94CBBE948BC6C9A2B9A" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="68502b0f0955ec7bc8f56677585c1c13">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="83b0043d-3627-4f29-99ea-ed882df73a05" xmlns:ns4="942c1815-1a1b-49ab-ae21-7a54e279a57b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7c7a778c7ed535cdadc2c6f960a471d8" ns3:_="" ns4:_="">
     <xsd:import namespace="83b0043d-3627-4f29-99ea-ed882df73a05"/>
@@ -11993,12 +12030,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80E629FC-C0A0-418E-A068-5110321EDDA0}">
   <ds:schemaRefs>
@@ -12008,6 +12039,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CEB0DF-FBF6-4FAC-A4B6-1450ADA239FD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12024,13 +12064,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updates and improved open_edd.py functionality
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2119" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{284E4E9F-0F49-4B79-B546-AE8650EB9B22}"/>
+  <xr:revisionPtr revIDLastSave="2122" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8000BA42-45A8-461E-B5CE-345E3C37BC45}"/>
   <bookViews>
-    <workbookView xWindow="2550" yWindow="2895" windowWidth="21600" windowHeight="11295" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="2550" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2243" uniqueCount="812">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2246" uniqueCount="812">
   <si>
     <t>Durham</t>
   </si>
@@ -8407,6 +8407,9 @@
       <c r="H29" s="9" t="s">
         <v>741</v>
       </c>
+      <c r="J29" t="s">
+        <v>529</v>
+      </c>
       <c r="K29">
         <v>396166</v>
       </c>
@@ -8439,6 +8442,9 @@
       <c r="H30" s="9" t="s">
         <v>496</v>
       </c>
+      <c r="J30" t="s">
+        <v>529</v>
+      </c>
       <c r="K30">
         <v>402042</v>
       </c>
@@ -8938,6 +8944,9 @@
       </c>
       <c r="H46" s="9" t="s">
         <v>417</v>
+      </c>
+      <c r="J46" t="s">
+        <v>529</v>
       </c>
       <c r="K46">
         <v>379385</v>
@@ -11885,12 +11894,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100125872C61801B94CBBE948BC6C9A2B9A" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="68502b0f0955ec7bc8f56677585c1c13">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="83b0043d-3627-4f29-99ea-ed882df73a05" xmlns:ns4="942c1815-1a1b-49ab-ae21-7a54e279a57b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7c7a778c7ed535cdadc2c6f960a471d8" ns3:_="" ns4:_="">
     <xsd:import namespace="83b0043d-3627-4f29-99ea-ed882df73a05"/>
@@ -12107,6 +12110,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80E629FC-C0A0-418E-A068-5110321EDDA0}">
   <ds:schemaRefs>
@@ -12116,15 +12125,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CEB0DF-FBF6-4FAC-A4B6-1450ADA239FD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12141,4 +12141,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
updates and bug fix
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2122" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8000BA42-45A8-461E-B5CE-345E3C37BC45}"/>
+  <xr:revisionPtr revIDLastSave="2124" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{852E849B-B9AF-4D88-B046-EAA555B0D14C}"/>
   <bookViews>
-    <workbookView xWindow="2550" yWindow="2895" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="960" yWindow="585" windowWidth="24825" windowHeight="13935" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -2446,9 +2446,6 @@
     <t>H:\BRWM\Remediation Division\Sites\Portland\Portland Harbor Dredge Project</t>
   </si>
   <si>
-    <t>SP Harbor Dredge</t>
-  </si>
-  <si>
     <t>L2656748-01</t>
   </si>
   <si>
@@ -2474,6 +2471,9 @@
   </si>
   <si>
     <t>L2643968</t>
+  </si>
+  <si>
+    <t>Harbor Dredge</t>
   </si>
 </sst>
 </file>
@@ -6995,7 +6995,7 @@
         <v>588</v>
       </c>
       <c r="B121" s="30" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>388</v>
@@ -7054,7 +7054,7 @@
         <v>783</v>
       </c>
       <c r="K122" s="23" t="s">
-        <v>804</v>
+        <v>803</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
@@ -7094,10 +7094,10 @@
         <v>584</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>807</v>
+        <v>806</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
       <c r="D124" s="34"/>
       <c r="E124" s="4" t="s">
@@ -7119,7 +7119,7 @@
         <v>783</v>
       </c>
       <c r="K124" s="23" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
@@ -7127,10 +7127,10 @@
         <v>413</v>
       </c>
       <c r="B125" s="30" t="s">
+        <v>807</v>
+      </c>
+      <c r="C125" s="3" t="s">
         <v>808</v>
-      </c>
-      <c r="C125" s="3" t="s">
-        <v>809</v>
       </c>
       <c r="D125" s="34"/>
       <c r="E125" s="4" t="s">
@@ -7152,7 +7152,7 @@
         <v>783</v>
       </c>
       <c r="K125" s="23" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
@@ -7160,10 +7160,10 @@
         <v>413</v>
       </c>
       <c r="B126" s="30" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D126" s="34"/>
       <c r="E126" s="4" t="s">
@@ -7185,7 +7185,7 @@
         <v>783</v>
       </c>
       <c r="K126" s="23" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
@@ -10813,7 +10813,7 @@
         <v>800</v>
       </c>
       <c r="C105" s="13" t="s">
-        <v>802</v>
+        <v>811</v>
       </c>
       <c r="D105" t="s">
         <v>88</v>

</xml_diff>

<commit_message>
xy point functinoaluity in bg_info
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2124" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{852E849B-B9AF-4D88-B046-EAA555B0D14C}"/>
+  <xr:revisionPtr revIDLastSave="2143" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61C2FF2F-381E-472F-82C8-0FD1B25A45E6}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="585" windowWidth="24825" windowHeight="13935" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="1755" yWindow="2400" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2246" uniqueCount="812">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2260" uniqueCount="816">
   <si>
     <t>Durham</t>
   </si>
@@ -2185,9 +2185,6 @@
     <t>Collins</t>
   </si>
   <si>
-    <t>H:\BRWM\PFAS - LD 1600\Sites\Brunswick\Henshaw-Lemaistre_007712 (EGAD 29532)</t>
-  </si>
-  <si>
     <t>Blaisdell</t>
   </si>
   <si>
@@ -2474,6 +2471,21 @@
   </si>
   <si>
     <t>Harbor Dredge</t>
+  </si>
+  <si>
+    <t>H:\BRWM\PFAS - LD 1600\Sites\Brunswick\Henshaw-Lemaistre_007712 (EGAD 28307)</t>
+  </si>
+  <si>
+    <t>16North</t>
+  </si>
+  <si>
+    <t>Russell</t>
+  </si>
+  <si>
+    <t>H:\BRWM\PFAS - LD 1600\Sites\Brunswick\Russell 00-W159 (NO EGAD)</t>
+  </si>
+  <si>
+    <t>C:\Users\Lucas.Beem\OneDrive - State of Maine\Documents\sites\pfas\cumberland_gray</t>
   </si>
 </sst>
 </file>
@@ -3463,7 +3475,7 @@
         <v>100</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="D11" s="34">
         <v>45747</v>
@@ -4199,7 +4211,7 @@
         <v>78</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="D34" s="34">
         <v>45845</v>
@@ -4231,7 +4243,7 @@
         <v>79</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="D35" s="34">
         <v>45845</v>
@@ -6316,7 +6328,7 @@
         <v>709</v>
       </c>
       <c r="B100" s="30" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>634</v>
@@ -6512,7 +6524,7 @@
         <v>706</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D106" s="34">
         <v>46135</v>
@@ -6544,7 +6556,7 @@
         <v>707</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D107" s="34">
         <v>46135</v>
@@ -6605,7 +6617,7 @@
         <v>65</v>
       </c>
       <c r="B109" s="30" t="s">
-        <v>720</v>
+        <v>719</v>
       </c>
       <c r="C109" s="3" t="s">
         <v>69</v>
@@ -6629,10 +6641,10 @@
         <v>7</v>
       </c>
       <c r="J109" s="40" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="K109" s="23" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
     </row>
     <row r="110" spans="1:11" x14ac:dyDescent="0.25">
@@ -6672,7 +6684,7 @@
         <v>641</v>
       </c>
       <c r="B111" s="30" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="C111" s="3" t="s">
         <v>638</v>
@@ -6704,7 +6716,7 @@
         <v>72</v>
       </c>
       <c r="B112" s="30" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>71</v>
@@ -6736,10 +6748,10 @@
         <v>710</v>
       </c>
       <c r="B113" s="30" t="s">
+        <v>717</v>
+      </c>
+      <c r="C113" s="3" t="s">
         <v>718</v>
-      </c>
-      <c r="C113" s="3" t="s">
-        <v>719</v>
       </c>
       <c r="D113" s="34">
         <v>46147</v>
@@ -6757,13 +6769,13 @@
         <v>7</v>
       </c>
       <c r="I113" s="40" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="J113" s="40" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="K113" s="23" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.25">
@@ -6771,7 +6783,7 @@
         <v>620</v>
       </c>
       <c r="B114" s="30" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>622</v>
@@ -6803,7 +6815,7 @@
         <v>641</v>
       </c>
       <c r="B115" s="30" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>638</v>
@@ -6832,10 +6844,10 @@
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
+        <v>767</v>
+      </c>
+      <c r="B116" s="30" t="s">
         <v>768</v>
-      </c>
-      <c r="B116" s="30" t="s">
-        <v>769</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>384</v>
@@ -6867,7 +6879,7 @@
         <v>641</v>
       </c>
       <c r="B117" s="30" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>638</v>
@@ -6891,7 +6903,7 @@
         <v>7</v>
       </c>
       <c r="J117" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
@@ -6899,7 +6911,7 @@
         <v>641</v>
       </c>
       <c r="B118" s="30" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="C118" s="3" t="s">
         <v>638</v>
@@ -6923,7 +6935,7 @@
         <v>7</v>
       </c>
       <c r="J118" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
@@ -6931,10 +6943,10 @@
         <v>641</v>
       </c>
       <c r="B119" s="30" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="D119" s="34">
         <v>46237</v>
@@ -6955,7 +6967,7 @@
         <v>7</v>
       </c>
       <c r="J119" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
@@ -6963,10 +6975,10 @@
         <v>641</v>
       </c>
       <c r="B120" s="30" t="s">
-        <v>781</v>
+        <v>780</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="D120" s="34">
         <v>46237</v>
@@ -6987,7 +6999,7 @@
         <v>7</v>
       </c>
       <c r="J120" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
@@ -6995,7 +7007,7 @@
         <v>588</v>
       </c>
       <c r="B121" s="30" t="s">
-        <v>802</v>
+        <v>801</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>388</v>
@@ -7016,10 +7028,10 @@
         <v>7</v>
       </c>
       <c r="I121" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="J121" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
@@ -7027,10 +7039,10 @@
         <v>588</v>
       </c>
       <c r="B122" s="30" t="s">
-        <v>796</v>
+        <v>795</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="D122" s="34">
         <v>46262</v>
@@ -7048,13 +7060,13 @@
         <v>7</v>
       </c>
       <c r="I122" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="J122" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="K122" s="23" t="s">
-        <v>803</v>
+        <v>802</v>
       </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.25">
@@ -7062,10 +7074,10 @@
         <v>22</v>
       </c>
       <c r="B123" s="30" t="s">
+        <v>793</v>
+      </c>
+      <c r="C123" s="3" t="s">
         <v>794</v>
-      </c>
-      <c r="C123" s="3" t="s">
-        <v>795</v>
       </c>
       <c r="D123" s="34">
         <v>46247</v>
@@ -7094,32 +7106,34 @@
         <v>584</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>806</v>
+        <v>805</v>
       </c>
       <c r="C124" s="3" t="s">
+        <v>803</v>
+      </c>
+      <c r="D124" s="34" t="s">
+        <v>782</v>
+      </c>
+      <c r="E124" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="F124" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="G124" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="H124" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="I124" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="J124" s="4" t="s">
+        <v>782</v>
+      </c>
+      <c r="K124" s="23" t="s">
         <v>804</v>
-      </c>
-      <c r="D124" s="34"/>
-      <c r="E124" s="4" t="s">
-        <v>783</v>
-      </c>
-      <c r="F124" s="4" t="s">
-        <v>783</v>
-      </c>
-      <c r="G124" s="4" t="s">
-        <v>783</v>
-      </c>
-      <c r="H124" s="4" t="s">
-        <v>783</v>
-      </c>
-      <c r="I124" s="4" t="s">
-        <v>783</v>
-      </c>
-      <c r="J124" s="4" t="s">
-        <v>783</v>
-      </c>
-      <c r="K124" s="23" t="s">
-        <v>805</v>
       </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
@@ -7127,32 +7141,34 @@
         <v>413</v>
       </c>
       <c r="B125" s="30" t="s">
+        <v>806</v>
+      </c>
+      <c r="C125" s="3" t="s">
         <v>807</v>
       </c>
-      <c r="C125" s="3" t="s">
-        <v>808</v>
-      </c>
-      <c r="D125" s="34"/>
+      <c r="D125" s="34" t="s">
+        <v>782</v>
+      </c>
       <c r="E125" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="G125" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="H125" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="I125" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="J125" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="K125" s="23" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
@@ -7160,39 +7176,50 @@
         <v>413</v>
       </c>
       <c r="B126" s="30" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>809</v>
-      </c>
-      <c r="D126" s="34"/>
+        <v>808</v>
+      </c>
+      <c r="D126" s="34" t="s">
+        <v>782</v>
+      </c>
       <c r="E126" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="G126" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="H126" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="I126" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="J126" s="4" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="K126" s="23" t="s">
-        <v>805</v>
+        <v>804</v>
       </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A127" s="3"/>
+      <c r="A127" s="3" t="s">
+        <v>65</v>
+      </c>
       <c r="B127" s="30"/>
-      <c r="D127" s="34"/>
-      <c r="E127" s="4"/>
+      <c r="C127" s="3" t="s">
+        <v>812</v>
+      </c>
+      <c r="D127" s="34">
+        <v>46288</v>
+      </c>
+      <c r="E127" s="4" t="s">
+        <v>7</v>
+      </c>
       <c r="F127" s="4"/>
       <c r="G127" s="4"/>
       <c r="H127" s="4"/>
@@ -7441,7 +7468,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L105"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -8405,7 +8432,7 @@
         <v>279</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="J29" t="s">
         <v>529</v>
@@ -9240,7 +9267,7 @@
         <v>464</v>
       </c>
       <c r="D55" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="E55" t="s">
         <v>360</v>
@@ -9810,7 +9837,7 @@
         <v>709</v>
       </c>
       <c r="D73" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="E73" t="s">
         <v>119</v>
@@ -9950,7 +9977,7 @@
         <v>127</v>
       </c>
       <c r="F77" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G77" s="11" t="s">
         <v>658</v>
@@ -9985,7 +10012,7 @@
         <v>127</v>
       </c>
       <c r="F78" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G78" s="11" t="s">
         <v>662</v>
@@ -10020,7 +10047,7 @@
         <v>127</v>
       </c>
       <c r="F79" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G79" s="11" t="s">
         <v>661</v>
@@ -10055,7 +10082,7 @@
         <v>127</v>
       </c>
       <c r="F80" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G80" s="11" t="s">
         <v>664</v>
@@ -10090,7 +10117,7 @@
         <v>127</v>
       </c>
       <c r="F81" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G81" s="11" t="s">
         <v>665</v>
@@ -10125,7 +10152,7 @@
         <v>127</v>
       </c>
       <c r="F82" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G82" s="11" t="s">
         <v>666</v>
@@ -10154,7 +10181,7 @@
         <v>671</v>
       </c>
       <c r="D83" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="E83" t="s">
         <v>225</v>
@@ -10166,7 +10193,7 @@
         <v>673</v>
       </c>
       <c r="H83" s="9" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="K83">
         <v>373564</v>
@@ -10285,13 +10312,13 @@
         <v>127</v>
       </c>
       <c r="F87" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G87" s="11" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="H87" s="9" t="s">
-        <v>715</v>
+        <v>811</v>
       </c>
       <c r="K87">
         <v>417730</v>
@@ -10317,10 +10344,10 @@
         <v>127</v>
       </c>
       <c r="F88" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="G88" s="11" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="H88" s="9" t="s">
         <v>711</v>
@@ -10340,7 +10367,7 @@
         <v>438</v>
       </c>
       <c r="C89" s="13" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="D89" t="s">
         <v>88</v>
@@ -10352,7 +10379,7 @@
         <v>455</v>
       </c>
       <c r="H89" s="9" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="J89" t="s">
         <v>529</v>
@@ -10372,19 +10399,19 @@
         <v>224</v>
       </c>
       <c r="C90" s="13" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="D90" t="s">
+        <v>724</v>
+      </c>
+      <c r="E90" t="s">
         <v>725</v>
       </c>
-      <c r="E90" t="s">
+      <c r="F90" t="s">
         <v>726</v>
       </c>
-      <c r="F90" t="s">
+      <c r="H90" s="11" t="s">
         <v>727</v>
-      </c>
-      <c r="H90" s="11" t="s">
-        <v>728</v>
       </c>
       <c r="K90">
         <v>395766</v>
@@ -10401,10 +10428,10 @@
         <v>670</v>
       </c>
       <c r="C91" s="13" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="D91" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E91" t="s">
         <v>225</v>
@@ -10413,7 +10440,7 @@
         <v>672</v>
       </c>
       <c r="H91" s="9" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="K91">
         <v>370364</v>
@@ -10430,10 +10457,10 @@
         <v>670</v>
       </c>
       <c r="C92" s="13" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="D92" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="E92" t="s">
         <v>225</v>
@@ -10442,7 +10469,7 @@
         <v>672</v>
       </c>
       <c r="H92" s="9" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="K92">
         <v>369839</v>
@@ -10459,7 +10486,7 @@
         <v>635</v>
       </c>
       <c r="C93" s="13" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="D93" t="s">
         <v>88</v>
@@ -10471,10 +10498,10 @@
         <v>455</v>
       </c>
       <c r="G93" s="11" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="H93" s="9" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="K93">
         <v>386078</v>
@@ -10488,7 +10515,7 @@
         <v>28947</v>
       </c>
       <c r="B94" s="17" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="C94" s="17" t="s">
         <v>449</v>
@@ -10503,10 +10530,10 @@
         <v>455</v>
       </c>
       <c r="G94" s="11" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="H94" s="9" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="K94">
         <v>368660</v>
@@ -10523,7 +10550,7 @@
         <v>203</v>
       </c>
       <c r="C95" s="13" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="D95" t="s">
         <v>88</v>
@@ -10532,13 +10559,13 @@
         <v>127</v>
       </c>
       <c r="F95" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="G95" s="11" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="H95" s="9" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="K95">
         <v>383498</v>
@@ -10555,7 +10582,7 @@
         <v>203</v>
       </c>
       <c r="C96" s="13" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="D96" t="s">
         <v>88</v>
@@ -10564,13 +10591,13 @@
         <v>127</v>
       </c>
       <c r="F96" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="G96" s="11" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="H96" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="K96">
         <v>381140</v>
@@ -10584,10 +10611,10 @@
         <v>29331</v>
       </c>
       <c r="B97" s="17" t="s">
+        <v>747</v>
+      </c>
+      <c r="C97" s="13" t="s">
         <v>748</v>
-      </c>
-      <c r="C97" s="13" t="s">
-        <v>749</v>
       </c>
       <c r="D97" t="s">
         <v>88</v>
@@ -10599,7 +10626,7 @@
         <v>455</v>
       </c>
       <c r="H97" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="J97" t="s">
         <v>529</v>
@@ -10619,7 +10646,7 @@
         <v>635</v>
       </c>
       <c r="C98" s="13" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="D98" t="s">
         <v>88</v>
@@ -10628,13 +10655,13 @@
         <v>127</v>
       </c>
       <c r="F98" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="G98" s="11" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
       <c r="H98" s="9" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="K98">
         <v>384636</v>
@@ -10651,7 +10678,7 @@
         <v>438</v>
       </c>
       <c r="C99" s="13" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="D99" t="s">
         <v>88</v>
@@ -10660,10 +10687,10 @@
         <v>127</v>
       </c>
       <c r="F99" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="H99" s="9" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="K99">
         <v>352211</v>
@@ -10680,7 +10707,7 @@
         <v>670</v>
       </c>
       <c r="C100" s="13" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="D100" t="s">
         <v>88</v>
@@ -10692,7 +10719,7 @@
         <v>672</v>
       </c>
       <c r="H100" s="9" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="K100">
         <v>372038</v>
@@ -10706,19 +10733,19 @@
         <v>64926</v>
       </c>
       <c r="B101" s="17" t="s">
+        <v>783</v>
+      </c>
+      <c r="C101" s="13" t="s">
+        <v>786</v>
+      </c>
+      <c r="D101" s="41" t="s">
         <v>784</v>
-      </c>
-      <c r="C101" s="13" t="s">
-        <v>787</v>
-      </c>
-      <c r="D101" s="41" t="s">
-        <v>785</v>
       </c>
       <c r="E101" t="s">
         <v>338</v>
       </c>
       <c r="H101" s="9" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
@@ -10729,7 +10756,7 @@
         <v>227</v>
       </c>
       <c r="C102" s="13" t="s">
-        <v>790</v>
+        <v>789</v>
       </c>
       <c r="D102" t="s">
         <v>88</v>
@@ -10738,10 +10765,13 @@
         <v>127</v>
       </c>
       <c r="F102" t="s">
-        <v>757</v>
+        <v>756</v>
+      </c>
+      <c r="G102" s="11" t="s">
+        <v>815</v>
       </c>
       <c r="H102" s="9" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="K102">
         <v>400597</v>
@@ -10755,19 +10785,19 @@
         <v>88</v>
       </c>
       <c r="B103" s="17" t="s">
+        <v>790</v>
+      </c>
+      <c r="C103" s="13" t="s">
         <v>791</v>
       </c>
-      <c r="C103" s="13" t="s">
+      <c r="D103" t="s">
+        <v>88</v>
+      </c>
+      <c r="E103" t="s">
+        <v>725</v>
+      </c>
+      <c r="F103" t="s">
         <v>792</v>
-      </c>
-      <c r="D103" t="s">
-        <v>88</v>
-      </c>
-      <c r="E103" t="s">
-        <v>726</v>
-      </c>
-      <c r="F103" t="s">
-        <v>793</v>
       </c>
       <c r="K103">
         <v>395950</v>
@@ -10781,10 +10811,10 @@
         <v>29148</v>
       </c>
       <c r="B104" s="17" t="s">
+        <v>796</v>
+      </c>
+      <c r="C104" s="13" t="s">
         <v>797</v>
-      </c>
-      <c r="C104" s="13" t="s">
-        <v>798</v>
       </c>
       <c r="D104" t="s">
         <v>88</v>
@@ -10793,10 +10823,10 @@
         <v>127</v>
       </c>
       <c r="F104" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
       <c r="I104" s="9" t="s">
-        <v>799</v>
+        <v>798</v>
       </c>
       <c r="K104">
         <v>399074</v>
@@ -10810,10 +10840,10 @@
         <v>88</v>
       </c>
       <c r="B105" s="17" t="s">
-        <v>800</v>
+        <v>799</v>
       </c>
       <c r="C105" s="13" t="s">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="D105" t="s">
         <v>88</v>
@@ -10825,7 +10855,36 @@
         <v>456</v>
       </c>
       <c r="I105" s="9" t="s">
-        <v>801</v>
+        <v>800</v>
+      </c>
+    </row>
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>88</v>
+      </c>
+      <c r="B106" s="17" t="s">
+        <v>712</v>
+      </c>
+      <c r="C106" s="13" t="s">
+        <v>813</v>
+      </c>
+      <c r="D106" t="s">
+        <v>88</v>
+      </c>
+      <c r="E106" t="s">
+        <v>127</v>
+      </c>
+      <c r="F106" t="s">
+        <v>756</v>
+      </c>
+      <c r="I106" s="9" t="s">
+        <v>814</v>
+      </c>
+      <c r="K106">
+        <v>419832</v>
+      </c>
+      <c r="L106">
+        <v>4864010</v>
       </c>
     </row>
   </sheetData>
@@ -11371,7 +11430,7 @@
         <v>399</v>
       </c>
       <c r="C17" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="D17" t="s">
         <v>307</v>
@@ -11793,7 +11852,7 @@
         <v>639</v>
       </c>
       <c r="E30" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="F30" t="s">
         <v>642</v>
@@ -11894,6 +11953,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100125872C61801B94CBBE948BC6C9A2B9A" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="68502b0f0955ec7bc8f56677585c1c13">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="83b0043d-3627-4f29-99ea-ed882df73a05" xmlns:ns4="942c1815-1a1b-49ab-ae21-7a54e279a57b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7c7a778c7ed535cdadc2c6f960a471d8" ns3:_="" ns4:_="">
     <xsd:import namespace="83b0043d-3627-4f29-99ea-ed882df73a05"/>
@@ -12110,12 +12175,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80E629FC-C0A0-418E-A068-5110321EDDA0}">
   <ds:schemaRefs>
@@ -12125,6 +12184,15 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CEB0DF-FBF6-4FAC-A4B6-1450ADA239FD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12141,13 +12209,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
town search in egad.py
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2143" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61C2FF2F-381E-472F-82C8-0FD1B25A45E6}"/>
+  <xr:revisionPtr revIDLastSave="2154" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99336B6A-1A7F-4111-A736-F5713E1A2178}"/>
   <bookViews>
-    <workbookView xWindow="1755" yWindow="2400" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="2970" yWindow="3180" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2260" uniqueCount="816">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2268" uniqueCount="822">
   <si>
     <t>Durham</t>
   </si>
@@ -2486,6 +2486,24 @@
   </si>
   <si>
     <t>C:\Users\Lucas.Beem\OneDrive - State of Maine\Documents\sites\pfas\cumberland_gray</t>
+  </si>
+  <si>
+    <t>unc</t>
+  </si>
+  <si>
+    <t>Olsky</t>
+  </si>
+  <si>
+    <t>Mayhew</t>
+  </si>
+  <si>
+    <t>H:\BRWM\Remediation Division\Sites\Mexico\Boise Cascade (Olsky)</t>
+  </si>
+  <si>
+    <t>REM00718</t>
+  </si>
+  <si>
+    <t>C:\Users\Lucas.Beem\OneDrive - State of Maine\Documents\sites\unc\olsky</t>
   </si>
 </sst>
 </file>
@@ -7468,7 +7486,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -10885,6 +10903,38 @@
       </c>
       <c r="L106">
         <v>4864010</v>
+      </c>
+    </row>
+    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>88</v>
+      </c>
+      <c r="B107" s="17" t="s">
+        <v>657</v>
+      </c>
+      <c r="C107" s="13" t="s">
+        <v>817</v>
+      </c>
+      <c r="D107" t="s">
+        <v>820</v>
+      </c>
+      <c r="E107" t="s">
+        <v>816</v>
+      </c>
+      <c r="F107" t="s">
+        <v>818</v>
+      </c>
+      <c r="G107" s="11" t="s">
+        <v>821</v>
+      </c>
+      <c r="I107" s="9" t="s">
+        <v>819</v>
+      </c>
+      <c r="K107">
+        <v>380083</v>
+      </c>
+      <c r="L107">
+        <v>4933678</v>
       </c>
     </row>
   </sheetData>
@@ -11953,12 +12003,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100125872C61801B94CBBE948BC6C9A2B9A" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="68502b0f0955ec7bc8f56677585c1c13">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="83b0043d-3627-4f29-99ea-ed882df73a05" xmlns:ns4="942c1815-1a1b-49ab-ae21-7a54e279a57b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7c7a778c7ed535cdadc2c6f960a471d8" ns3:_="" ns4:_="">
     <xsd:import namespace="83b0043d-3627-4f29-99ea-ed882df73a05"/>
@@ -12175,6 +12219,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80E629FC-C0A0-418E-A068-5110321EDDA0}">
   <ds:schemaRefs>
@@ -12184,15 +12234,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04CEB0DF-FBF6-4FAC-A4B6-1450ADA239FD}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12209,4 +12250,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED9CEC6D-B35B-412B-B4C7-0CC920F4535C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
minor updates and corrections
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2154" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99336B6A-1A7F-4111-A736-F5713E1A2178}"/>
+  <xr:revisionPtr revIDLastSave="2165" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A970060B-D002-48A2-BD5F-F4F7FCAA8FBD}"/>
   <bookViews>
-    <workbookView xWindow="2970" yWindow="3180" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="-25965" yWindow="2010" windowWidth="21600" windowHeight="11160" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2268" uniqueCount="822">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2276" uniqueCount="826">
   <si>
     <t>Durham</t>
   </si>
@@ -2482,9 +2482,6 @@
     <t>Russell</t>
   </si>
   <si>
-    <t>H:\BRWM\PFAS - LD 1600\Sites\Brunswick\Russell 00-W159 (NO EGAD)</t>
-  </si>
-  <si>
     <t>C:\Users\Lucas.Beem\OneDrive - State of Maine\Documents\sites\pfas\cumberland_gray</t>
   </si>
   <si>
@@ -2504,6 +2501,21 @@
   </si>
   <si>
     <t>C:\Users\Lucas.Beem\OneDrive - State of Maine\Documents\sites\unc\olsky</t>
+  </si>
+  <si>
+    <t>L2662765</t>
+  </si>
+  <si>
+    <t>Currie</t>
+  </si>
+  <si>
+    <t>Pamco</t>
+  </si>
+  <si>
+    <t>H:\BRWM\Remediation Division\Sites\Auburn\Pamco Machine Company, 100 washington street</t>
+  </si>
+  <si>
+    <t>H:\BRWM\PFAS - LD 1600\Sites\Brunswick\Russell 00-W159 (164446)</t>
   </si>
 </sst>
 </file>
@@ -7228,7 +7240,9 @@
       <c r="A127" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B127" s="30"/>
+      <c r="B127" s="30" t="s">
+        <v>821</v>
+      </c>
       <c r="C127" s="3" t="s">
         <v>812</v>
       </c>
@@ -7486,7 +7500,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -10786,7 +10800,7 @@
         <v>756</v>
       </c>
       <c r="G102" s="11" t="s">
-        <v>815</v>
+        <v>814</v>
       </c>
       <c r="H102" s="9" t="s">
         <v>788</v>
@@ -10896,7 +10910,7 @@
         <v>756</v>
       </c>
       <c r="I106" s="9" t="s">
-        <v>814</v>
+        <v>825</v>
       </c>
       <c r="K106">
         <v>419832</v>
@@ -10913,28 +10927,51 @@
         <v>657</v>
       </c>
       <c r="C107" s="13" t="s">
+        <v>816</v>
+      </c>
+      <c r="D107" t="s">
+        <v>819</v>
+      </c>
+      <c r="E107" t="s">
+        <v>815</v>
+      </c>
+      <c r="F107" t="s">
         <v>817</v>
       </c>
-      <c r="D107" t="s">
+      <c r="G107" s="11" t="s">
         <v>820</v>
       </c>
-      <c r="E107" t="s">
-        <v>816</v>
-      </c>
-      <c r="F107" t="s">
+      <c r="I107" s="9" t="s">
         <v>818</v>
-      </c>
-      <c r="G107" s="11" t="s">
-        <v>821</v>
-      </c>
-      <c r="I107" s="9" t="s">
-        <v>819</v>
       </c>
       <c r="K107">
         <v>380083</v>
       </c>
       <c r="L107">
         <v>4933678</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>88</v>
+      </c>
+      <c r="B108" s="17" t="s">
+        <v>747</v>
+      </c>
+      <c r="C108" s="13" t="s">
+        <v>823</v>
+      </c>
+      <c r="D108" t="s">
+        <v>88</v>
+      </c>
+      <c r="E108" t="s">
+        <v>360</v>
+      </c>
+      <c r="F108" t="s">
+        <v>822</v>
+      </c>
+      <c r="H108" s="9" t="s">
+        <v>824</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove replaced pfas_table files
</commit_message>
<xml_diff>
--- a/lookup/Spill_lab_tracking.xlsx
+++ b/lookup/Spill_lab_tracking.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateofmaine-my.sharepoint.com/personal/lucas_beem_maine_gov/Documents/Documents/refactor/lookup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2171" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB06F432-12CE-423E-9D25-5F73DE09C2BD}"/>
+  <xr:revisionPtr revIDLastSave="2196" documentId="13_ncr:1_{4923A7FC-61C1-43DD-ACDC-2AD5F26F4CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EEF5691F-A0A6-4A03-8A09-A2FC6C2CC113}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="2730" windowWidth="21600" windowHeight="11295" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{8A7E386D-9303-4138-8E00-F12B91A17E09}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2281" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2288" uniqueCount="831">
   <si>
     <t>Durham</t>
   </si>
@@ -2516,6 +2516,21 @@
   </si>
   <si>
     <t>L2662765-01</t>
+  </si>
+  <si>
+    <t>REM03779</t>
+  </si>
+  <si>
+    <t>C:\Users\Lucas.Beem\OneDrive - State of Maine\Documents\sites\vrap\Pamco_and_mobile</t>
+  </si>
+  <si>
+    <t>H:\BRWM\Remediation Division\Sites\Auburn\Washington Street Mobil</t>
+  </si>
+  <si>
+    <t>REM03777</t>
+  </si>
+  <si>
+    <t>Washington Mobile</t>
   </si>
 </sst>
 </file>
@@ -7510,7 +7525,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05C0069-E32D-47E3-8952-41BB91A7FDEB}">
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L110"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
@@ -10962,8 +10977,8 @@
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
-        <v>88</v>
+      <c r="A108">
+        <v>38753</v>
       </c>
       <c r="B108" s="17" t="s">
         <v>747</v>
@@ -10972,7 +10987,7 @@
         <v>822</v>
       </c>
       <c r="D108" t="s">
-        <v>88</v>
+        <v>826</v>
       </c>
       <c r="E108" t="s">
         <v>360</v>
@@ -10980,9 +10995,54 @@
       <c r="F108" t="s">
         <v>821</v>
       </c>
+      <c r="G108" s="11" t="s">
+        <v>827</v>
+      </c>
       <c r="H108" s="9" t="s">
         <v>823</v>
       </c>
+      <c r="K108">
+        <v>401415</v>
+      </c>
+      <c r="L108">
+        <v>4882256</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A109">
+        <v>28815</v>
+      </c>
+      <c r="B109" s="17" t="s">
+        <v>747</v>
+      </c>
+      <c r="C109" s="13" t="s">
+        <v>830</v>
+      </c>
+      <c r="D109" t="s">
+        <v>829</v>
+      </c>
+      <c r="E109" t="s">
+        <v>360</v>
+      </c>
+      <c r="F109" t="s">
+        <v>821</v>
+      </c>
+      <c r="G109" s="11" t="s">
+        <v>827</v>
+      </c>
+      <c r="H109" s="9" t="s">
+        <v>828</v>
+      </c>
+      <c r="K109">
+        <v>401450</v>
+      </c>
+      <c r="L109">
+        <v>4882404</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B110" s="17"/>
+      <c r="C110" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>